<commit_message>
chore: ignore all modality data paths in .gitignore
</commit_message>
<xml_diff>
--- a/replica/data/handwriting/PaHaw Dataset/PaHaW_files/corpus_PaHaW.xlsx
+++ b/replica/data/handwriting/PaHaw Dataset/PaHaW_files/corpus_PaHaW.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0e0e6fefce8cdbfd/Attachments/Desktop/Homework/Projects in BME AI/Project_biomed_AI/Enhancing-Multimodal-Parkinsons-Disease-Classification-and-Explainability/replica/data/handwriting/PaHaw Dataset/PaHaW_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_D61DCE1FAC2F98B2F839C5E3E2F15D6E73244F28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04E348D6-AC4A-461F-A3C7-59DB1FFFE5B6}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_D61DCE1FAC2F98B2F839C5E3E2F15D6E73244F28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18644E19-D205-4609-80CA-B5D10CB956A7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="150000" iterateDelta="1E-4" concurrentCalc="0"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
@@ -368,6 +370,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2627,4 +2633,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C1B8189-ED07-44D8-8596-DC021D6AFEE3}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>